<commit_message>
Add image of assembled board
</commit_message>
<xml_diff>
--- a/PM5644/PM8547_20/Docs/BOM_8547_20.xlsx
+++ b/PM5644/PM8547_20/Docs/BOM_8547_20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\PTV_Preservation\PM5644\PM8547_20\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\PTV_Preservation\PM5644\PM8547_20\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDCE33F9-FFEB-4A78-B0DA-A601C430351E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12F85C3-0BDE-43EC-B0AD-392291E89F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9810" yWindow="2400" windowWidth="28590" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5025" yWindow="5025" windowWidth="28800" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="96">
   <si>
     <t>Reference</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>PCF84C00T</t>
+  </si>
+  <si>
+    <t>2K</t>
   </si>
 </sst>
 </file>
@@ -1103,7 +1106,7 @@
         <v>32</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="C36" t="s">
         <v>47</v>

</xml_diff>